<commit_message>
añade opcion para eliminar paquetes y corrige bug
</commit_message>
<xml_diff>
--- a/base de datos/manifiesto miami/manifiesto_miami_20_paquetes.xlsx
+++ b/base de datos/manifiesto miami/manifiesto_miami_20_paquetes.xlsx
@@ -167,15 +167,6 @@
     <t>cliente</t>
   </si>
   <si>
-    <t>largo (cm)</t>
-  </si>
-  <si>
-    <t>ancho (cm)</t>
-  </si>
-  <si>
-    <t>altura (cm)</t>
-  </si>
-  <si>
     <t>descripcion</t>
   </si>
   <si>
@@ -225,6 +216,15 @@
   </si>
   <si>
     <t>terrestre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">largo </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ancho </t>
+  </si>
+  <si>
+    <t>alto</t>
   </si>
 </sst>
 </file>
@@ -274,15 +274,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -582,42 +579,42 @@
         <v>45</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>46</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>64</v>
+      <c r="D2" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E2" s="2">
         <v>2.5</v>
@@ -631,22 +628,22 @@
       <c r="H2" s="2">
         <v>10</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>65</v>
+      <c r="D3" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E3" s="2">
         <v>1.2</v>
@@ -660,22 +657,22 @@
       <c r="H3" s="2">
         <v>8</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>66</v>
+      <c r="D4" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="E4" s="2">
         <v>5</v>
@@ -689,22 +686,22 @@
       <c r="H4" s="2">
         <v>15</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="B5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>64</v>
+      <c r="D5" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E5" s="2">
         <v>0.8</v>
@@ -718,22 +715,22 @@
       <c r="H5" s="2">
         <v>12</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" s="4" t="s">
+      <c r="B6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>65</v>
+      <c r="D6" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E6" s="2">
         <v>3.5</v>
@@ -747,22 +744,22 @@
       <c r="H6" s="2">
         <v>10</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="B7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>66</v>
+      <c r="D7" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="E7" s="2">
         <v>-2</v>
@@ -776,22 +773,22 @@
       <c r="H7" s="2">
         <v>15</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="B8" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>64</v>
+      <c r="D8" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E8" s="2">
         <v>0</v>
@@ -805,22 +802,22 @@
       <c r="H8" s="2">
         <v>10</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>65</v>
+      <c r="B9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>62</v>
       </c>
       <c r="E9" s="2">
         <v>2.4</v>
@@ -834,22 +831,22 @@
       <c r="H9" s="2">
         <v>12</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="B10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>66</v>
+      <c r="D10" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>18</v>
@@ -863,22 +860,22 @@
       <c r="H10" s="2">
         <v>15</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="B11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>64</v>
+      <c r="D11" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E11" s="2">
         <v>4.2</v>
@@ -892,22 +889,22 @@
       <c r="H11" s="2">
         <v>20</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C12" s="4" t="s">
+      <c r="B12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>65</v>
+      <c r="D12" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E12" s="2">
         <v>-1.5</v>
@@ -921,22 +918,22 @@
       <c r="H12" s="2">
         <v>15</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" s="4" t="s">
+      <c r="B13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>66</v>
+      <c r="D13" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="E13" s="2">
         <v>2.8</v>
@@ -950,22 +947,22 @@
       <c r="H13" s="2">
         <v>10</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="4" t="s">
+      <c r="B14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>64</v>
+      <c r="D14" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E14" s="2">
         <v>3.1</v>
@@ -979,22 +976,22 @@
       <c r="H14" s="2">
         <v>15</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="B15" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>65</v>
+      <c r="D15" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E15" s="2">
         <v>3.1</v>
@@ -1008,22 +1005,22 @@
       <c r="H15" s="2">
         <v>15</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="5" t="s">
+      <c r="B16" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>66</v>
+      <c r="D16" s="4" t="s">
+        <v>63</v>
       </c>
       <c r="E16" s="2">
         <v>6.2</v>
@@ -1037,22 +1034,22 @@
       <c r="H16" s="2">
         <v>20</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C17" s="4" t="s">
+      <c r="B17" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>64</v>
+      <c r="D17" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>29</v>
@@ -1066,22 +1063,22 @@
       <c r="H17" s="2">
         <v>12</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I17" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="4" t="s">
+      <c r="B18" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>65</v>
+      <c r="D18" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E18" s="2">
         <v>2.1</v>
@@ -1095,22 +1092,22 @@
       <c r="H18" s="2">
         <v>10</v>
       </c>
-      <c r="I18" s="5" t="s">
+      <c r="I18" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C19" s="4" t="s">
+      <c r="B19" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>66</v>
+      <c r="D19" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="E19" s="2">
         <v>-3</v>
@@ -1124,22 +1121,22 @@
       <c r="H19" s="2">
         <v>20</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="4" t="s">
+      <c r="B20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>64</v>
+      <c r="D20" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E20" s="2">
         <v>7.5</v>
@@ -1153,22 +1150,22 @@
       <c r="H20" s="2">
         <v>20</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="I20" s="3" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C21" s="4" t="s">
+      <c r="B21" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>65</v>
+      <c r="D21" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E21" s="2">
         <v>0</v>
@@ -1182,7 +1179,7 @@
       <c r="H21" s="2">
         <v>15</v>
       </c>
-      <c r="I21" s="4" t="s">
+      <c r="I21" s="3" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
corrige la api, cambia las variables de entorno y actualiza a la ultima version de la app
</commit_message>
<xml_diff>
--- a/base de datos/manifiesto miami/manifiesto_miami_20_paquetes.xlsx
+++ b/base de datos/manifiesto miami/manifiesto_miami_20_paquetes.xlsx
@@ -167,15 +167,6 @@
     <t>cliente</t>
   </si>
   <si>
-    <t>largo (cm)</t>
-  </si>
-  <si>
-    <t>ancho (cm)</t>
-  </si>
-  <si>
-    <t>altura (cm)</t>
-  </si>
-  <si>
     <t>descripcion</t>
   </si>
   <si>
@@ -225,6 +216,15 @@
   </si>
   <si>
     <t>terrestre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">largo </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ancho </t>
+  </si>
+  <si>
+    <t>alto</t>
   </si>
 </sst>
 </file>
@@ -274,15 +274,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -582,42 +579,42 @@
         <v>45</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>46</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>64</v>
+      <c r="D2" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E2" s="2">
         <v>2.5</v>
@@ -631,22 +628,22 @@
       <c r="H2" s="2">
         <v>10</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>65</v>
+      <c r="D3" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E3" s="2">
         <v>1.2</v>
@@ -660,22 +657,22 @@
       <c r="H3" s="2">
         <v>8</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>66</v>
+      <c r="D4" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="E4" s="2">
         <v>5</v>
@@ -689,22 +686,22 @@
       <c r="H4" s="2">
         <v>15</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C5" s="4" t="s">
+      <c r="B5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>64</v>
+      <c r="D5" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E5" s="2">
         <v>0.8</v>
@@ -718,22 +715,22 @@
       <c r="H5" s="2">
         <v>12</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" s="4" t="s">
+      <c r="B6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>65</v>
+      <c r="D6" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E6" s="2">
         <v>3.5</v>
@@ -747,22 +744,22 @@
       <c r="H6" s="2">
         <v>10</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="4" t="s">
+      <c r="B7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>66</v>
+      <c r="D7" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="E7" s="2">
         <v>-2</v>
@@ -776,22 +773,22 @@
       <c r="H7" s="2">
         <v>15</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="B8" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>64</v>
+      <c r="D8" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E8" s="2">
         <v>0</v>
@@ -805,22 +802,22 @@
       <c r="H8" s="2">
         <v>10</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>65</v>
+      <c r="B9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>62</v>
       </c>
       <c r="E9" s="2">
         <v>2.4</v>
@@ -834,22 +831,22 @@
       <c r="H9" s="2">
         <v>12</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="B10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>66</v>
+      <c r="D10" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>18</v>
@@ -863,22 +860,22 @@
       <c r="H10" s="2">
         <v>15</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C11" s="4" t="s">
+      <c r="B11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>64</v>
+      <c r="D11" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E11" s="2">
         <v>4.2</v>
@@ -892,22 +889,22 @@
       <c r="H11" s="2">
         <v>20</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C12" s="4" t="s">
+      <c r="B12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>65</v>
+      <c r="D12" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E12" s="2">
         <v>-1.5</v>
@@ -921,22 +918,22 @@
       <c r="H12" s="2">
         <v>15</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" s="4" t="s">
+      <c r="B13" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>66</v>
+      <c r="D13" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="E13" s="2">
         <v>2.8</v>
@@ -950,22 +947,22 @@
       <c r="H13" s="2">
         <v>10</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="4" t="s">
+      <c r="B14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>64</v>
+      <c r="D14" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E14" s="2">
         <v>3.1</v>
@@ -979,22 +976,22 @@
       <c r="H14" s="2">
         <v>15</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="B15" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>65</v>
+      <c r="D15" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E15" s="2">
         <v>3.1</v>
@@ -1008,22 +1005,22 @@
       <c r="H15" s="2">
         <v>15</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="5" t="s">
+      <c r="B16" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>66</v>
+      <c r="D16" s="4" t="s">
+        <v>63</v>
       </c>
       <c r="E16" s="2">
         <v>6.2</v>
@@ -1037,22 +1034,22 @@
       <c r="H16" s="2">
         <v>20</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C17" s="4" t="s">
+      <c r="B17" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>64</v>
+      <c r="D17" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>29</v>
@@ -1066,22 +1063,22 @@
       <c r="H17" s="2">
         <v>12</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I17" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="4" t="s">
+      <c r="B18" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>65</v>
+      <c r="D18" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E18" s="2">
         <v>2.1</v>
@@ -1095,22 +1092,22 @@
       <c r="H18" s="2">
         <v>10</v>
       </c>
-      <c r="I18" s="5" t="s">
+      <c r="I18" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C19" s="4" t="s">
+      <c r="B19" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>66</v>
+      <c r="D19" s="3" t="s">
+        <v>63</v>
       </c>
       <c r="E19" s="2">
         <v>-3</v>
@@ -1124,22 +1121,22 @@
       <c r="H19" s="2">
         <v>20</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="I19" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="4" t="s">
+      <c r="B20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>64</v>
+      <c r="D20" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="E20" s="2">
         <v>7.5</v>
@@ -1153,22 +1150,22 @@
       <c r="H20" s="2">
         <v>20</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="I20" s="3" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C21" s="4" t="s">
+      <c r="B21" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="4" t="s">
-        <v>65</v>
+      <c r="D21" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="E21" s="2">
         <v>0</v>
@@ -1182,7 +1179,7 @@
       <c r="H21" s="2">
         <v>15</v>
       </c>
-      <c r="I21" s="4" t="s">
+      <c r="I21" s="3" t="s">
         <v>36</v>
       </c>
     </row>

</xml_diff>